<commit_message>
Add external heartbeat monitor (healthchecks.io) for laptop power-off detection
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,22 @@
     <font>
       <b val="1"/>
       <sz val="20"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000AA00"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="3">
@@ -63,12 +79,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -550,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -613,6 +633,46 @@
         <is>
           <t>Overall DD %</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-02-18</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -707,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -717,6 +777,166 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>📊 ACCOUNT OVERVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Current Balance:</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>$6,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Initial Balance:</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$100,000.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total P&amp;L:</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Return:</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-94.00%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>📈 TRADING STATS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11"/>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Total Trades:</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wins:</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Losses:</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Win Rate:</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Avg Win:</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Avg Loss:</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>$0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Profit Factor:</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>Last Updated: 2026-02-19 03:00:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
FIX: Critical R variable bug + reduce 80-bar minimum to 30
Critical Bug Fixed:
- _manage_positions() external close path used undefined variable R
  causing NameError crash when any trade closes (SL/TP hit by broker)
- After 5 such crashes, bot would shut down permanently
- Fixed: use info['R'] (safe dict lookup) instead of bare R variable

Signal Window Fix:
- generate_signals() required 80 M1 bars before running (80 min)
- Combined with 60-min breakout window + 15-bar staleness limit,
  bot could only catch signals from last ~15 min of breakout window
- Reduced to 30 bars (15 ORB + 10 rolling avg + 5 buffer)
- Now catches breakouts from ~10:00 ET instead of ~10:30 ET
- Effective signal window: ~45 min instead of ~15 min (3x improvement)
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -672,6 +672,166 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -924,7 +1084,7 @@
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Last Updated: 2026-02-19 03:00:08</t>
+          <t>Last Updated: 2026-02-23 03:00:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CRITICAL FIX: fill_price=0.0 bug + PnL deal history retry
Root cause: MT5 result.price returns 0.0 for IOC fills on FundedNext-Server 2.
This caused entry=0 in tracked_positions, breaking BE trigger, trail SL,
slippage calc, journal entry, and Telegram notification.

First live trade (US2000 SELL 1.16 @ 2626.10) had to be emergency-closed
because trail SL never activated despite ~ profit (>1R). Actual result:
+.04 but logged as PnL=.00 due to deal history timing bug.

Fixes:
1. place_order(): Recover fill price from deal history with 0.3s delay
   when result.price=0.0. Ultimate fallback: use requested price.
2. _execute_signal(): Double-check fill_price, fallback to expected_price.
3. _get_closed_trade_pnl(): Retry 3x with 0.5s delay for deals to register.
4. Log annotated with emergency close reason and impact analysis.
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,22 +35,6 @@
     <font>
       <b val="1"/>
       <sz val="20"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="0000AA00"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="3">
@@ -79,16 +63,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -454,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:AN2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,77 +465,306 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Entry Price</t>
+          <t>Planned Entry</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Actual Entry</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Slippage Pts</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Slippage $</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Stop Loss</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>TP1</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>TP2</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>TP3</t>
-        </is>
-      </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>TP</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Lot Size</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Risk Amount</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>R (Risk Pts)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Planned RR</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Signal Time</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Fill Time</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Exec Delay (s)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>HTF Trend</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>ORB Range</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Exit Time</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Exit Reason</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>P&amp;L %</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Actual RR</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>MFE (pts)</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>MAE (pts)</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>MFE (R)</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>MAE (R)</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Time in Trade</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>BE Hit?</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Balance After</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>Drawdown %</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Spread Entry</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Spread Exit</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Exit Slip Pts</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Session</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Weekday</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>20:51:49</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>US2000</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2629.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>2637.3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2610.349999999999</v>
+      </c>
+      <c r="L2" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="M2" t="n">
+        <v>90</v>
+      </c>
+      <c r="N2" t="n">
+        <v>7.700000000000273</v>
+      </c>
+      <c r="O2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2026-02-23 17:06:00</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>20:51:49</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>13549.9</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>bearish</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>21:41:18</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>External/TP/SL</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>2629.1</v>
+      </c>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="n">
+        <v>341.44</v>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0h 49m</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AG2" t="n">
+        <v>6138.04</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>R=7.70 slip=+2626.10</t>
         </is>
       </c>
     </row>
@@ -570,7 +779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -633,206 +842,6 @@
         <is>
           <t>Overall DD %</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-02-18</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-02-20</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-02-21</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -927,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -937,166 +946,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>📊 ACCOUNT OVERVIEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="4"/>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Current Balance:</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>$6,000.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Initial Balance:</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>$100,000.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Total P&amp;L:</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Return:</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>-94.00%</t>
-        </is>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>📈 TRADING STATS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11"/>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Total Trades:</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Wins:</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Losses:</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Win Rate:</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Avg Win:</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Avg Loss:</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>$0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Profit Factor:</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>0.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Last Updated: 2026-02-23 03:00:00</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
FIX DATA: Correct Trade #1 journal with MT5 actual values
MT5 deal history confirmed:
  Entry: 2625.9 (was 0.0), Exit: 2614.0 (was 0.0)
  PnL: +\.04 (was \.00), RR: 1.55 (was 0)
  Slippage: 3.7 pts favorable (was 2626.1 pts)
  MFE: 11.9 pts / 1.55R, MAE: 0.31 pts / 0.04R
  Exec delay: 1.34s (was 13549.9s)

Also corrected: position_state.json daily_pnl, edge_guard.json trade record.
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -667,13 +667,13 @@
         <v>2629.6</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>2625.9</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>42.92</v>
       </c>
       <c r="J2" t="n">
         <v>2637.3</v>
@@ -695,16 +695,16 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-02-23 17:06:00</t>
+          <t>2026-02-23 20:51:44</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>20:51:49</t>
+          <t>20:51:45</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>13549.9</v>
+        <v>1.34</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
         <v>16.9</v>
       </c>
       <c r="U2" t="n">
-        <v>0</v>
+        <v>2614</v>
       </c>
       <c r="V2" t="inlineStr">
         <is>
@@ -724,27 +724,29 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>External/TP/SL</t>
+          <t>EMERGENCY_CLOSE (fill_price=0 bug)</t>
         </is>
       </c>
       <c r="X2" t="n">
-        <v>0</v>
+        <v>138.04</v>
       </c>
       <c r="Y2" t="n">
-        <v>0</v>
+        <v>2.301</v>
       </c>
       <c r="Z2" t="n">
-        <v>0</v>
+        <v>1.55</v>
       </c>
       <c r="AA2" t="n">
-        <v>0</v>
+        <v>11.9</v>
       </c>
       <c r="AB2" t="n">
-        <v>2629.1</v>
-      </c>
-      <c r="AC2" t="inlineStr"/>
+        <v>0.31</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>1.55</v>
+      </c>
       <c r="AD2" t="n">
-        <v>341.44</v>
+        <v>0.04</v>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
@@ -753,7 +755,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (bug prevented)</t>
         </is>
       </c>
       <c r="AG2" t="n">
@@ -764,8 +766,11 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>R=7.70 slip=+2626.10</t>
-        </is>
+          <t>R=7.70 slip=+3.70 entry=2625.9 exit=2614.0 | CORRECTED: fill_price=0.0 bug caused wrong values in original log</t>
+        </is>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
6-index backtest + strategy cleanup + trade reporting fixes
- Add US2000/SWI20 to run_3year_backtest.py (6 indices total)
- Clean up strategy_ict_clean.py: remove 10 dead compat params, add **_kwargs
- Revert lookback_ranges to 10 (tested 5/15, both worse)
- Fix SL/TP trade reporting: actual exit_price + specific exit_reason from MT5 deals
- Fix /emergency command: now records journal + telegram per position
- Fix _emergency_close_all: full exit details instead of exit_price=0
- New _get_closed_trade_details() method for MT5 deal history
- Backtest comparison metrics saved (OLD/NEW/LB5/LB15/SEED variants)
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -37,7 +37,7 @@
       <sz val="20"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
         <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -63,12 +75,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN2"/>
+  <dimension ref="A1:AN4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -771,6 +785,294 @@
       </c>
       <c r="AJ2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>14:24:54</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SWI20</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>13982.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>13981.65</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>-0.45</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J3" t="n">
+        <v>13974.6</v>
+      </c>
+      <c r="K3" t="n">
+        <v>14000.85</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="M3" t="n">
+        <v>92.0706</v>
+      </c>
+      <c r="N3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="O3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2026-02-26 10:39:00</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>14:24:54</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>13554.3</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>bullish</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>14:38:18</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>External/TP/SL</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0h 13m</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AG3" t="n">
+        <v>6091.77</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>R=7.50 slip=+0.00 spread=0 lat=221ms</t>
+        </is>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>20:48:35</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>US2000</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2626</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2625.3</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>-0.7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>21.91</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2628.4</v>
+      </c>
+      <c r="K4" t="n">
+        <v>2620</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3.13</v>
+      </c>
+      <c r="M4" t="n">
+        <v>91.37655000000001</v>
+      </c>
+      <c r="N4" t="n">
+        <v>2.400000000000091</v>
+      </c>
+      <c r="O4" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2026-02-27 17:03:00</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>20:48:35</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>13535.9</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>bearish</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>20:52:55</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>External/TP/SL</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>0h 4m</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AG4" t="n">
+        <v>5988.48</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>R=2.40 slip=+0.00 spread=0 lat=155ms</t>
+        </is>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Friday</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: P&L recording for broker-executed SL/TP closes
- Increased deal history retries: 3x0.5s -> 6x1.0s
- Widened lookback window: 1 day -> 7 days (fixes weekend edge case)
- Added deferred P&L re-query via background thread (10s + 30s retry)
- Added duplicate close guard in _manage_positions
- Corrected Trade #2 (SWI20) P&L: 0 -> -46.27
- Corrected Trade #3 (US2000) P&L: 0 -> -103.29
- True weekly P&L: -11.52 (was incorrectly showing +138.04)
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -863,7 +863,7 @@
         <v>39.3</v>
       </c>
       <c r="U3" t="n">
-        <v>0</v>
+        <v>13973.7</v>
       </c>
       <c r="V3" t="inlineStr">
         <is>
@@ -872,17 +872,17 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>External/TP/SL</t>
+          <t>SL Hit (reconstructed from balance)</t>
         </is>
       </c>
       <c r="X3" t="n">
-        <v>0</v>
+        <v>-46.27</v>
       </c>
       <c r="Y3" t="n">
-        <v>0</v>
+        <v>-0.754</v>
       </c>
       <c r="Z3" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="AA3" t="n">
         <v>4.65</v>
@@ -914,7 +914,7 @@
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>R=7.50 slip=+0.00 spread=0 lat=221ms</t>
+          <t>R=7.50 slip=+0.00 spread=0 lat=221ms | CORRECTED: P&amp;L was  due to deal history bug. Actual loss -.27 from balance delta 6138.04-&gt;6091.77</t>
         </is>
       </c>
       <c r="AJ3" t="n">
@@ -1007,7 +1007,7 @@
         <v>20.8</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>2628.6</v>
       </c>
       <c r="V4" t="inlineStr">
         <is>
@@ -1016,17 +1016,17 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>External/TP/SL</t>
+          <t>SL Hit (reconstructed from balance)</t>
         </is>
       </c>
       <c r="X4" t="n">
-        <v>0</v>
+        <v>-103.29</v>
       </c>
       <c r="Y4" t="n">
-        <v>0</v>
+        <v>-1.696</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>-1.13</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
@@ -1034,7 +1034,6 @@
       <c r="AB4" t="n">
         <v>2.2</v>
       </c>
-      <c r="AC4" t="inlineStr"/>
       <c r="AD4" t="n">
         <v>0.92</v>
       </c>
@@ -1056,14 +1055,12 @@
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>R=2.40 slip=+0.00 spread=0 lat=155ms</t>
+          <t>R=2.40 slip=+0.00 spread=0 lat=155ms | CORRECTED: P&amp;L was  due to deal history bug. Actual loss -.29 from balance delta 6091.77-&gt;5988.48</t>
         </is>
       </c>
       <c r="AJ4" t="n">
         <v>0</v>
       </c>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr">
         <is>
           <t>US</t>

</xml_diff>

<commit_message>
Add minimum R guard (5pts), fix edge guard PnL data, fix journal Trade #4 (US30)
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN4"/>
+  <dimension ref="A1:AN5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1069,6 +1069,150 @@
       <c r="AN4" t="inlineStr">
         <is>
           <t>Friday</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-03</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>21:26:23</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>US30</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>sell</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>47782.62</v>
+      </c>
+      <c r="G5" t="n">
+        <v>47759.09</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>-23.53</v>
+      </c>
+      <c r="I5" t="n">
+        <v>37.65</v>
+      </c>
+      <c r="J5" t="n">
+        <v>47811.12</v>
+      </c>
+      <c r="K5" t="n">
+        <v>47711.37</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="M5" t="n">
+        <v>89.82719999999999</v>
+      </c>
+      <c r="N5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2026-03-03 17:42:00</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>21:26:23</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>13463.7</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>bearish</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>311.45</v>
+      </c>
+      <c r="U5" t="n">
+        <v>47811.12</v>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>21:28:56</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="X5" s="4" t="n">
+        <v>-87.66</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>-2.535</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>-1.92</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>11.26</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>46.83</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>0h 2m</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AG5" t="n">
+        <v>5900.82</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>R=28.50 slip=+0.00 spread=0 lat=263ms</t>
+        </is>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix deal history symbol mismatch: balance-delta fallback when wrong-symbol deals returned
- mt5_connector: _get_closed_trade_details returns symbol_mismatch=True when filtered deals empty
- mt5_connector: position closure handler uses MT5 account balance delta as PnL fallback
- Infers exit_price from SL/TP based on PnL sign when deal data unreliable
- Corrected trade journal Trade #5 (NDX100): exit 25092.49, PnL -64.56, balance 5836.26
- Corrected edge guard Trade #5: PnL, RR, balance, equity curve
- Added new indices backtest (FRA40/UK100/HK50/JP225 - none viable)
- Added forex ORB backtest scripts and reports
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN5"/>
+  <dimension ref="A1:AN6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1213,6 +1213,150 @@
       <c r="AN5" t="inlineStr">
         <is>
           <t>Tuesday</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>20:43:22</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>NDX100</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>buy</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>25130.36</v>
+      </c>
+      <c r="G6" t="n">
+        <v>25119.54</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-10.82</v>
+      </c>
+      <c r="I6" t="n">
+        <v>25.97</v>
+      </c>
+      <c r="J6" t="n">
+        <v>25093.61</v>
+      </c>
+      <c r="K6" t="n">
+        <v>25222.235</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="M6" t="n">
+        <v>88.5123</v>
+      </c>
+      <c r="N6" t="n">
+        <v>36.75</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>2026-03-05 16:59:00</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>20:43:22</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>13462.5</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>bullish</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>139.53</v>
+      </c>
+      <c r="U6" t="n">
+        <v>25092.49</v>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>20:48:09</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>SL_HIT</t>
+        </is>
+      </c>
+      <c r="X6" s="4" t="n">
+        <v>-64.56</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>-1.094</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>21.19</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>0h 4m</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AG6" t="n">
+        <v>5836.26</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>R=36.75 slip=+0.00 spread=0 lat=163ms | CORRECTED: Exit was 25092.49 not 2628.4 (US2000 price). PnL=-64.56 not -190.95. MT5 deal history symbol mismatch bug.</t>
+        </is>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Thursday</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FROZEN: Production lock - ORB Clean v22, trail 0.5R, 6 indices, all audits passed
Strategy: ORB Clean Breakout (ICT) v22
Trail buffer: 0.5R (A/B tested vs 0.75R and 1.0R - winner)
Live indices: SPX500, NDX100, GER30, FRA40, US30, US2000
Backtest: 16yr HistData, 1212 trades, WR 66.9%, PF 1.57, Sharpe 2.20
FundedNext sim: 13/13 passes, 0 breaches
Live account: 13958231, running on FundedNext Stellar-2

DO NOT MODIFY without explicit approval.
</commit_message>
<xml_diff>
--- a/live/reports/trade_journal.xlsx
+++ b/live/reports/trade_journal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Trades" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Daily Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Weekly Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trades" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN6"/>
+  <dimension ref="A1:AQ6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -650,6 +650,21 @@
       <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Weekday</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>Commission</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>Swap</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>Risk Tier</t>
         </is>
       </c>
     </row>

</xml_diff>